<commit_message>
Use spilled arrays in excel.
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_asianoptions.xlsx
+++ b/tests/workbooktests/workbooks/test_asianoptions.xlsx
@@ -1,36 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA8B2AF-B533-47F6-BD25-CCA42C3A57B9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F34E64-4E99-47F7-8FDB-A9CD0F4DC124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{826B86DD-8849-449F-936D-EDB49B97704B}"/>
+    <workbookView xWindow="-4560" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{826B86DD-8849-449F-936D-EDB49B97704B}"/>
   </bookViews>
   <sheets>
     <sheet name="Market data" sheetId="1" r:id="rId1"/>
     <sheet name="ContinuousAveragingAsianOption" sheetId="2" r:id="rId2"/>
     <sheet name="DiscreteAveragingAsianOption" sheetId="3" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId4"/>
-  </externalReferences>
   <definedNames>
     <definedName name="BlackVolatility">'Market data'!$B$7</definedName>
     <definedName name="DiscountCurve">'Market data'!$B$4</definedName>
     <definedName name="DividendCurve">'Market data'!$B$5</definedName>
     <definedName name="EvaluationDate">'Market data'!$B$2</definedName>
-    <definedName name="InitialValueS0">'[1]Market data'!$B$9</definedName>
+    <definedName name="InitialValueS0">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -39,6 +47,28 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="83">
   <si>
@@ -298,7 +328,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -367,55 +397,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Market data"/>
-      <sheetName val="Calculators"/>
-      <sheetName val="DeltaVolQuote"/>
-      <sheetName val="Vanilla &amp; Forward options"/>
-      <sheetName val="Cash dividend engines"/>
-      <sheetName val="American option engines"/>
-      <sheetName val="Quanto options"/>
-      <sheetName val="Multi-asset options"/>
-      <sheetName val="Other options"/>
-      <sheetName val="Heston engines"/>
-      <sheetName val="Heston-Hull-White engines"/>
-      <sheetName val="Binomial tree engine"/>
-      <sheetName val="Finite Difference engines"/>
-      <sheetName val="Monte Carlo engines"/>
-      <sheetName val="QD engines"/>
-      <sheetName val="Other engines"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="9">
-          <cell r="B9">
-            <v>100</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -736,13 +717,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{175C4B6A-2FF6-4E41-A92B-A67BBE399B16}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -750,43 +731,43 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="e">
-        <f t="array" aca="1" ref="B2" ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="B2" s="1">
+        <f t="array" ref="B2">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="e">
-        <f ca="1">_xll.qlFlatForward(B2,0.03,"actual365fixed")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="B4" t="str">
+        <f>_xll.qlFlatForward(B2,0.03,"actual365fixed")</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R4C2YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" t="e">
-        <f ca="1">_xll.qlFlatForward(B2,0.02,"actual365fixed")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="B5" t="str">
+        <f>_xll.qlFlatForward(B2,0.02,"actual365fixed")</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R5C2YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
-      <c r="B7" t="e">
-        <f t="array" aca="1" ref="B7" ca="1">_xll.qlBlackConstantVol(EvaluationDate,"NullCalendar",0.25,"Act/365")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="B7" t="str">
+        <f t="array" ref="B7">_xll.qlBlackConstantVol(EvaluationDate,"NullCalendar",0.25,"Act/365")</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R7C2BlackVolTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -794,16 +775,16 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B10" t="e">
-        <f t="array" aca="1" ref="B10" ca="1">_xll.qlGeneralizedBlackScholesProcess(B9,DividendCurve,DiscountCurve,BlackVolatility)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
+      <c r="B10" t="str">
+        <f t="array" ref="B10">_xll.qlGeneralizedBlackScholesProcess(B9,DividendCurve,DiscountCurve,BlackVolatility)</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R10C2GeneralizedBlackScholesProcess,A</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -811,7 +792,7 @@
         <v>0.19504877171446253</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -819,7 +800,7 @@
         <v>0.39716005835063128</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -827,7 +808,7 @@
         <v>7.5903860839074258E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -835,7 +816,7 @@
         <v>1.3901714719854346</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -843,7 +824,7 @@
         <v>-0.3506856326404631</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -851,13 +832,13 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="2" t="e">
-        <f t="array" aca="1" ref="B18" ca="1">_xll.qlHestonProcess(DiscountCurve,DividendCurve,InitialValueS0,B12,B13,B14,B15,B16,B17)</f>
-        <v>#VALUE!</v>
+      <c r="B18" s="2" t="str" cm="1">
+        <f t="array" ref="B18">_xll.qlHestonProcess(DiscountCurve,DividendCurve,B9,B12,B13,B14,B15,B16,B17)</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R18C2HestonProcess,A</v>
       </c>
     </row>
   </sheetData>
@@ -868,27 +849,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01E8CF31-6A5D-416B-9E37-822AFE48B67A}">
   <dimension ref="A1:B49"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.75" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="1" t="e">
-        <f ca="1">EvaluationDate</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+      <c r="B1" s="1">
+        <f>EvaluationDate</f>
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -896,34 +877,34 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="2" t="e">
-        <f t="array" aca="1" ref="B5" ca="1">_xll.qlPlainVanillaPayoff("Call", 100)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="B5" s="2" t="str">
+        <f t="array" ref="B5">_xll.qlPlainVanillaPayoff("Call", 100)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R5C2PlainVanillaPayoff,A</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="e">
-        <f t="array" aca="1" ref="B6" ca="1">_xll.qlEuropeanExercise($B$1+365)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="B6" s="2" t="str">
+        <f t="array" ref="B6">_xll.qlEuropeanExercise($B$1+365)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R6C2EuropeanExercise,A</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2" t="e">
-        <f t="array" aca="1" ref="B7" ca="1">_xll.qlContinuousAveragingAsianOption(B4,B5,B6,$B$1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="B7" s="2" t="str">
+        <f t="array" ref="B7">_xll.qlContinuousAveragingAsianOption(B4,B5,B6,$B$1)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R7C2ContinuousAveragingAsianOption,A</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -931,43 +912,43 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="1" t="e">
-        <f ca="1">$B$1</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
+      <c r="B10" s="1">
+        <f>$B$1</f>
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="2" t="e">
-        <f t="array" aca="1" ref="B11" ca="1">_xll.qlPlainVanillaPayoff("Call", 100)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
+      <c r="B11" s="2" t="str">
+        <f t="array" ref="B11">_xll.qlPlainVanillaPayoff("Call", 100)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R11C2PlainVanillaPayoff,A</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="2" t="e">
-        <f t="array" aca="1" ref="B12" ca="1">_xll.qlEuropeanExercise($B$1+365)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
+      <c r="B12" s="2" t="str">
+        <f t="array" ref="B12">_xll.qlEuropeanExercise($B$1+365)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R12C2EuropeanExercise,A</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="2" t="e">
-        <f t="array" aca="1" ref="B13" ca="1">_xll.qlContinuousAveragingAsianOptionWithStartDate(B9,B10,B11,B12,$B$1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
+      <c r="B13" s="2" t="str">
+        <f t="array" ref="B13">_xll.qlContinuousAveragingAsianOptionWithStartDate(B9,B10,B11,B12,$B$1)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R13C2ContinuousAveragingAsianOption,A</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -975,34 +956,34 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="2" t="e">
-        <f t="array" aca="1" ref="B17" ca="1">_xll.qlPlainVanillaPayoff("Call", 100)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
+      <c r="B17" s="2" t="str">
+        <f t="array" ref="B17">_xll.qlPlainVanillaPayoff("Call", 100)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R17C2PlainVanillaPayoff,A</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="2" t="e">
-        <f t="array" aca="1" ref="B18" ca="1">_xll.qlEuropeanExercise($B$1+365)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
+      <c r="B18" s="2" t="str">
+        <f t="array" ref="B18">_xll.qlEuropeanExercise($B$1+365)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R18C2EuropeanExercise,A</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="2" t="e">
-        <f t="array" aca="1" ref="B19" ca="1">_xll.qlContinuousAveragingAsianOption(B16,B17,B18,$B$1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
+      <c r="B19" s="2" t="str">
+        <f t="array" ref="B19">_xll.qlContinuousAveragingAsianOption(B16,B17,B18,$B$1)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R19C2ContinuousAveragingAsianOption,A</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>7</v>
       </c>
@@ -1010,79 +991,79 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="1" t="e">
-        <f ca="1">$B$1</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
+      <c r="B22" s="1">
+        <f>$B$1</f>
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="2" t="e">
-        <f t="array" aca="1" ref="B23" ca="1">_xll.qlPlainVanillaPayoff("Call", 100)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
+      <c r="B23" s="2" t="str">
+        <f t="array" ref="B23">_xll.qlPlainVanillaPayoff("Call", 100)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R23C2PlainVanillaPayoff,A</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
-      <c r="B24" s="2" t="e">
-        <f t="array" aca="1" ref="B24" ca="1">_xll.qlEuropeanExercise($B$1+365)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
+      <c r="B24" s="2" t="str">
+        <f t="array" ref="B24">_xll.qlEuropeanExercise($B$1+365)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R24C2EuropeanExercise,A</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="2" t="e">
-        <f t="array" aca="1" ref="B25" ca="1">_xll.qlContinuousAveragingAsianOptionWithStartDate(B21,B22,B23,B24,$B$1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2">
+      <c r="B25" s="2" t="str">
+        <f t="array" ref="B25">_xll.qlContinuousAveragingAsianOptionWithStartDate(B21,B22,B23,B24,$B$1)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R25C2ContinuousAveragingAsianOption,A</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>25</v>
       </c>
-      <c r="B28" t="e">
-        <f ca="1">'Market data'!$B$10</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2">
+      <c r="B28" t="str">
+        <f>'Market data'!$B$10</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R10C2GeneralizedBlackScholesProcess,A</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>23</v>
       </c>
-      <c r="B29" t="e">
-        <f t="array" aca="1" ref="B29" ca="1">_xll.qlAnalyticContinuousGeometricAveragePriceAsianEngine(B28,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2">
+      <c r="B29" t="str">
+        <f t="array" ref="B29">_xll.qlAnalyticContinuousGeometricAveragePriceAsianEngine(B28,B1)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R29C2AnalyticContinuousGeometricAveragePriceAsianEngine,A</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="4" t="e">
-        <f t="array" aca="1" ref="B30" ca="1">_xll.qlInstrumentNPV($B$7,_xll.qlInstrumentSetPricingEngine($B$7,B29))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
+      <c r="B30" s="4">
+        <f t="array" ref="B30">_xll.qlInstrumentNPV($B$7,_xll.qlInstrumentSetPricingEngine($B$7,B29))</f>
+        <v>5.5725238097120151</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>25</v>
       </c>
-      <c r="B32" t="e">
-        <f ca="1">'Market data'!$B$18</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2">
+      <c r="B32" t="str">
+        <f>'Market data'!$B$18</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R18C2HestonProcess,A</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -1090,7 +1071,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -1098,34 +1079,34 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>28</v>
       </c>
-      <c r="B35" t="e">
-        <f t="array" aca="1" ref="B35" ca="1">_xll.qlAnalyticContinuousGeometricAveragePriceAsianHestonEngine(B32,B33,B34,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
+      <c r="B35" t="str">
+        <f t="array" ref="B35">_xll.qlAnalyticContinuousGeometricAveragePriceAsianHestonEngine(B32,B33,B34,B1)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R35C2AnalyticContinuousGeometricAveragePriceAsianHestonEngine,A</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="4" t="e">
-        <f t="array" aca="1" ref="B36" ca="1">_xll.qlInstrumentNPV($B$7,_xll.qlInstrumentSetPricingEngine($B$7,B35))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2">
+      <c r="B36" s="4">
+        <f t="array" ref="B36">_xll.qlInstrumentNPV($B$7,_xll.qlInstrumentSetPricingEngine($B$7,B35))</f>
+        <v>7.8889590093712725</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>25</v>
       </c>
-      <c r="B39" t="e">
-        <f ca="1">'Market data'!$B$10</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2">
+      <c r="B39" t="str">
+        <f>'Market data'!$B$10</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R10C2GeneralizedBlackScholesProcess,A</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>29</v>
       </c>
@@ -1133,25 +1114,25 @@
         <v>100</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>30</v>
       </c>
-      <c r="B41" t="e">
-        <f t="array" aca="1" ref="B41" ca="1">_xll.qlContinuousArithmeticAsianLevyEngine(B39,B40,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2">
+      <c r="B41" t="str">
+        <f t="array" ref="B41">_xll.qlContinuousArithmeticAsianLevyEngine(B39,B40,B1)</f>
+        <v>欣[test_asianoptions.xlsx]ContinuousAveragingAsianOption!R41C2ContinuousArithmeticAsianLevyEngine,A</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>24</v>
       </c>
-      <c r="B42" s="4" t="e">
-        <f t="array" aca="1" ref="B42" ca="1">_xll.qlInstrumentNPV($B$25,_xll.qlInstrumentSetPricingEngine($B$25,B41))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="49" spans="2:2">
+      <c r="B42" s="4">
+        <f t="array" ref="B42">_xll.qlInstrumentNPV($B$25,_xll.qlInstrumentSetPricingEngine($B$25,B41))</f>
+        <v>5.865545937685539</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" s="4"/>
     </row>
   </sheetData>
@@ -1162,50 +1143,50 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F905595E-E751-4C88-8FF3-5AD27AC5A197}">
   <dimension ref="A1:E113"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="48.125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="5" t="e">
-        <f ca="1">EvaluationDate</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="B1" s="5">
+        <f>EvaluationDate</f>
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" s="5"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
       <c r="B3" s="5"/>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="5" t="e">
-        <f ca="1">B1-182</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="B4" s="5">
+        <f>B1-182</f>
+        <v>45992</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="5" t="e">
-        <f ca="1">B1+365</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="B5" s="5">
+        <f>B1+365</f>
+        <v>46539</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -1213,19 +1194,19 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="2" t="e">
-        <f t="array" aca="1" ref="B7" ca="1">_xll.qlMakeSchedule(B4,B5,B6)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="B7" s="2" t="str">
+        <f t="array" ref="B7">_xll.qlMakeSchedule(B4,B5,B6)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R7C2Schedule,A</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8" s="5"/>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -1234,160 +1215,142 @@
       </c>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="1" t="e">
-        <f t="array" aca="1" ref="A10:A28" ca="1">_xll.qlScheduleDates(B7)</f>
-        <v>#VALUE!</v>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" cm="1">
+        <f t="array" ref="A10:A28">_xll.qlScheduleDates(B7)</f>
+        <v>45992</v>
       </c>
       <c r="B10" s="2">
         <v>100</v>
       </c>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>46023</v>
       </c>
       <c r="B11" s="2">
         <v>100</v>
       </c>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>46054</v>
       </c>
       <c r="B12" s="2">
         <v>100</v>
       </c>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>46082</v>
       </c>
       <c r="B13" s="2">
         <v>100</v>
       </c>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>46113</v>
       </c>
       <c r="B14" s="2">
         <v>100</v>
       </c>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>46143</v>
       </c>
       <c r="B15" s="2">
         <v>100</v>
       </c>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>46174</v>
       </c>
       <c r="B16" s="2">
         <v>100</v>
       </c>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>46204</v>
       </c>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>46235</v>
       </c>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>46266</v>
       </c>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>46296</v>
       </c>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>46327</v>
       </c>
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>46357</v>
       </c>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>46388</v>
       </c>
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>46419</v>
       </c>
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>46447</v>
       </c>
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>46478</v>
       </c>
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>46508</v>
       </c>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="1" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>46539</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>7</v>
       </c>
@@ -1395,34 +1358,34 @@
         <v>14</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="2" t="e">
-        <f t="array" aca="1" ref="B32" ca="1">_xll.qlPlainVanillaPayoff("Call", 100)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2">
+      <c r="B32" s="2" t="str">
+        <f t="array" ref="B32">_xll.qlPlainVanillaPayoff("Call", 100)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R32C2PlainVanillaPayoff,A</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>10</v>
       </c>
-      <c r="B33" s="2" t="e">
-        <f t="array" aca="1" ref="B33" ca="1">_xll.qlEuropeanExercise($A$28)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2">
+      <c r="B33" s="2" t="str">
+        <f t="array" ref="B33">_xll.qlEuropeanExercise($A$28)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R33C2EuropeanExercise,A</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>45</v>
       </c>
-      <c r="B34" s="2" t="e">
-        <f t="array" aca="1" ref="B34" ca="1">_xll.qlDiscreteAveragingAsianOption(B31,_xlfn.ANCHORARRAY(A10),B32,B33,$B$10:$B$16,$B$1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
+      <c r="B34" s="2" t="str">
+        <f t="array" ref="B34">_xll.qlDiscreteAveragingAsianOption(B31,_xlfn.ANCHORARRAY(A10),B32,B33,$B$10:$B$16,$B$1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R34C2DiscreteAveragingAsianOption,A</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>7</v>
       </c>
@@ -1430,70 +1393,70 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>9</v>
       </c>
-      <c r="B37" s="2" t="e">
-        <f t="array" aca="1" ref="B37" ca="1">_xll.qlPlainVanillaPayoff("Call", 100)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
+      <c r="B37" s="2" t="str">
+        <f t="array" ref="B37">_xll.qlPlainVanillaPayoff("Call", 100)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R37C2PlainVanillaPayoff,A</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="2" t="e">
-        <f t="array" aca="1" ref="B38" ca="1">_xll.qlEuropeanExercise($A$28)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2">
+      <c r="B38" s="2" t="str">
+        <f t="array" ref="B38">_xll.qlEuropeanExercise($A$28)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R38C2EuropeanExercise,A</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>45</v>
       </c>
-      <c r="B39" s="2" t="e">
-        <f t="array" aca="1" ref="B39" ca="1">_xll.qlDiscreteAveragingAsianOption(B36,_xlfn.ANCHORARRAY(A10),B37,B38,$B$10:$B$16,$B$1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2">
+      <c r="B39" s="2" t="str">
+        <f t="array" ref="B39">_xll.qlDiscreteAveragingAsianOption(B36,_xlfn.ANCHORARRAY(A10),B37,B38,$B$10:$B$16,$B$1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R39C2DiscreteAveragingAsianOption,A</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="2" t="e">
-        <f ca="1">'Market data'!$B$10</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2">
+      <c r="B42" s="2" t="str">
+        <f>'Market data'!$B$10</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R10C2GeneralizedBlackScholesProcess,A</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>46</v>
       </c>
-      <c r="B43" s="2" t="e">
-        <f t="array" aca="1" ref="B43" ca="1">_xll.qlAnalyticDiscreteGeometricAveragePriceAsianEngine(B42,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2">
+      <c r="B43" s="2" t="str">
+        <f t="array" ref="B43">_xll.qlAnalyticDiscreteGeometricAveragePriceAsianEngine(B42,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R43C2AnalyticDiscreteGeometricAveragePriceAsianEngine,A</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>24</v>
       </c>
-      <c r="B44" s="6" t="e">
-        <f t="array" aca="1" ref="B44" ca="1">_xll.qlInstrumentNPV($B$34,_xll.qlInstrumentSetPricingEngine($B$34,B43))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2">
+      <c r="B44" s="6">
+        <f t="array" ref="B44">_xll.qlInstrumentNPV($B$34,_xll.qlInstrumentSetPricingEngine($B$34,B43))</f>
+        <v>3.624243093201974</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>25</v>
       </c>
-      <c r="B46" s="2" t="e">
-        <f ca="1">'Market data'!$B$18</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2">
+      <c r="B46" s="2" t="str">
+        <f>'Market data'!$B$18</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R18C2HestonProcess,A</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>27</v>
       </c>
@@ -1501,70 +1464,70 @@
         <v>100</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="2" t="e">
-        <f t="array" aca="1" ref="B48" ca="1">_xll.qlAnalyticDiscreteGeometricAveragePriceAsianHestonEngine(B46,B47,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2">
+      <c r="B48" s="2" t="str">
+        <f t="array" ref="B48">_xll.qlAnalyticDiscreteGeometricAveragePriceAsianHestonEngine(B46,B47,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R48C2AnalyticDiscreteGeometricAveragePriceAsianHestonEngine,A</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>24</v>
       </c>
-      <c r="B49" s="6" t="e">
-        <f t="array" aca="1" ref="B49" ca="1">_xll.qlInstrumentNPV($B$34,_xll.qlInstrumentSetPricingEngine($B$34,B48))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2">
+      <c r="B49" s="6">
+        <f t="array" ref="B49">_xll.qlInstrumentNPV($B$34,_xll.qlInstrumentSetPricingEngine($B$34,B48))</f>
+        <v>5.0152940452426105</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>45</v>
       </c>
-      <c r="B51" s="2" t="e">
-        <f t="array" aca="1" ref="B51" ca="1">_xll.qlDiscreteAveragingAsianOption(B31,A16:A28,B32,B33,,$B$1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2">
+      <c r="B51" s="2" t="str">
+        <f t="array" ref="B51">_xll.qlDiscreteAveragingAsianOption(B31,A16:A28,B32,B33,,$B$1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R51C2DiscreteAveragingAsianOption,A</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>25</v>
       </c>
-      <c r="B52" s="2" t="e">
-        <f ca="1">'Market data'!$B$10</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
+      <c r="B52" s="2" t="str">
+        <f>'Market data'!$B$10</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R10C2GeneralizedBlackScholesProcess,A</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>48</v>
       </c>
-      <c r="B53" s="2" t="e">
-        <f t="array" aca="1" ref="B53" ca="1">_xll.qlAnalyticDiscreteGeometricAverageStrikeAsianEngine(B52,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2">
+      <c r="B53" s="2" t="str">
+        <f t="array" ref="B53">_xll.qlAnalyticDiscreteGeometricAverageStrikeAsianEngine(B52,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R53C2AnalyticDiscreteGeometricAverageStrikeAsianEngine,A</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>24</v>
       </c>
-      <c r="B54" s="6" t="e">
-        <f t="array" aca="1" ref="B54" ca="1">_xll.qlInstrumentNPV($B$51,_xll.qlInstrumentSetPricingEngine($B$51,B53))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2">
+      <c r="B54" s="6">
+        <f t="array" ref="B54">_xll.qlInstrumentNPV($B$51,_xll.qlInstrumentSetPricingEngine($B$51,B53))</f>
+        <v>6.0276403042264377</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>25</v>
       </c>
-      <c r="B57" s="2" t="e">
-        <f ca="1">'Market data'!$B$10</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
+      <c r="B57" s="2" t="str">
+        <f>'Market data'!$B$10</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R10C2GeneralizedBlackScholesProcess,A</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>33</v>
       </c>
@@ -1572,7 +1535,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="59" spans="1:2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>34</v>
       </c>
@@ -1580,7 +1543,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>35</v>
       </c>
@@ -1588,34 +1551,34 @@
         <v>50</v>
       </c>
     </row>
-    <row r="61" spans="1:2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>36</v>
       </c>
-      <c r="B61" s="2" t="e">
-        <f t="array" aca="1" ref="B61" ca="1">_xll.qlFdBlackScholesAsianEngine(B57,B58,B59,B60,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2">
+      <c r="B61" s="2" t="str">
+        <f t="array" ref="B61">_xll.qlFdBlackScholesAsianEngine(B57,B58,B59,B60,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R61C2FdBlackScholesAsianEngine,A</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>24</v>
       </c>
-      <c r="B62" s="6" t="e">
-        <f t="array" aca="1" ref="B62" ca="1">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B61))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4">
+      <c r="B62" s="6">
+        <f t="array" ref="B62">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B61))</f>
+        <v>3.9825557394734163</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>25</v>
       </c>
-      <c r="B65" s="2" t="e">
-        <f ca="1">'Market data'!$B$10</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4">
+      <c r="B65" s="2" t="str">
+        <f>'Market data'!$B$10</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R10C2GeneralizedBlackScholesProcess,A</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>49</v>
       </c>
@@ -1623,7 +1586,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:4">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>51</v>
       </c>
@@ -1631,69 +1594,69 @@
         <v>10</v>
       </c>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>50</v>
       </c>
-      <c r="B68" s="2" t="e">
-        <f t="array" aca="1" ref="B68" ca="1">_xll.qlChoiAsianEngine(B65,B66,B67)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4">
+      <c r="B68" s="2" t="str">
+        <f t="array" ref="B68">_xll.qlChoiAsianEngine(B65,B66,B67)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R68C2ChoiAsianEngine,A</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>24</v>
       </c>
-      <c r="B69" s="6" t="e">
-        <f t="array" aca="1" ref="B69" ca="1">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B68))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4">
+      <c r="B69" s="6">
+        <f t="array" ref="B69">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B68))</f>
+        <v>3.904737756175467</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>25</v>
       </c>
-      <c r="B71" s="2" t="e">
-        <f ca="1">'Market data'!$B$10</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4">
+      <c r="B71" s="2" t="str">
+        <f>'Market data'!$B$10</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R10C2GeneralizedBlackScholesProcess,A</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>52</v>
       </c>
-      <c r="B72" s="2" t="e">
-        <f t="array" aca="1" ref="B72" ca="1">_xll.qlTurnbullWakemanAsianEngine(B71,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4">
+      <c r="B72" s="2" t="str">
+        <f t="array" ref="B72">_xll.qlTurnbullWakemanAsianEngine(B71,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R72C2TurnbullWakemanAsianEngine,A</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>24</v>
       </c>
-      <c r="B73" s="6" t="e">
-        <f t="array" aca="1" ref="B73" ca="1">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B72))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="15">
+      <c r="B73" s="6">
+        <f t="array" ref="B73">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B72))</f>
+        <v>3.9472649968721769</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="77" spans="1:4">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>25</v>
       </c>
-      <c r="B77" s="2" t="e">
-        <f ca="1">'Market data'!$B$10</f>
-        <v>#VALUE!</v>
+      <c r="B77" s="2" t="str">
+        <f>'Market data'!$B$10</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R10C2GeneralizedBlackScholesProcess,A</v>
       </c>
       <c r="D77" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="78" spans="1:4">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>53</v>
       </c>
@@ -1704,7 +1667,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="79" spans="1:4">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>57</v>
       </c>
@@ -1712,7 +1675,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="80" spans="1:4">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>59</v>
       </c>
@@ -1720,7 +1683,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="81" spans="1:4">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>61</v>
       </c>
@@ -1728,7 +1691,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="82" spans="1:4">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>63</v>
       </c>
@@ -1739,7 +1702,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="83" spans="1:4">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>65</v>
       </c>
@@ -1747,7 +1710,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="84" spans="1:4">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>67</v>
       </c>
@@ -1755,7 +1718,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="85" spans="1:4">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>69</v>
       </c>
@@ -1766,78 +1729,78 @@
         <v>70</v>
       </c>
     </row>
-    <row r="87" spans="1:4">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>71</v>
       </c>
-      <c r="B87" s="2" t="e">
-        <f t="array" aca="1" ref="B87" ca="1">_xll.qlMCDiscreteArithmeticAPEngine(B77,B78,,,,B82,,,B85,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4">
+      <c r="B87" s="2" t="str">
+        <f t="array" ref="B87">_xll.qlMCDiscreteArithmeticAPEngine(B77,B78,,,,B82,,,B85,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R87C2MCLDDiscreteArithmeticAPEngine,A</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>24</v>
       </c>
-      <c r="B88" s="6" t="e">
-        <f t="array" aca="1" ref="B88" ca="1">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B87))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4">
+      <c r="B88" s="6">
+        <f t="array" ref="B88">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B87))</f>
+        <v>3.9276917312830051</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>72</v>
       </c>
-      <c r="B89" s="2" t="e">
-        <f t="array" aca="1" ref="B89" ca="1">_xll.qlMCDiscreteArithmeticASEngine(B77,B78,,,B82,,,B85,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4">
+      <c r="B89" s="2" t="str">
+        <f t="array" ref="B89">_xll.qlMCDiscreteArithmeticASEngine(B77,B78,,,B82,,,B85,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R89C2MCLDDiscreteArithmeticASEngine,A</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>24</v>
       </c>
-      <c r="B90" s="6" t="e">
-        <f t="array" aca="1" ref="B90" ca="1">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B89))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4">
+      <c r="B90" s="6">
+        <f t="array" ref="B90">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B89))</f>
+        <v>6.704804858255164</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>74</v>
       </c>
-      <c r="B92" s="2" t="e">
-        <f t="array" aca="1" ref="B92" ca="1">_xll.qlMCDiscreteGeometricAPEngine(B77,B78,,,B82,,,B85,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4">
+      <c r="B92" s="2" t="str">
+        <f t="array" ref="B92">_xll.qlMCDiscreteGeometricAPEngine(B77,B78,,,B82,,,B85,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R92C2MCLDDiscreteGeometricAPEngine,A</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>24</v>
       </c>
-      <c r="B93" s="6" t="e">
-        <f t="array" aca="1" ref="B93" ca="1">_xll.qlInstrumentNPV($B$34,_xll.qlInstrumentSetPricingEngine($B$34,B92))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="15">
+      <c r="B93" s="6">
+        <f t="array" ref="B93">_xll.qlInstrumentNPV($B$34,_xll.qlInstrumentSetPricingEngine($B$34,B92))</f>
+        <v>3.6326393112176851</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="98" spans="1:4">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>25</v>
       </c>
-      <c r="B98" s="2" t="e">
-        <f ca="1">'Market data'!B18</f>
-        <v>#VALUE!</v>
+      <c r="B98" s="2" t="str">
+        <f>'Market data'!B18</f>
+        <v>欣[test_asianoptions.xlsx]Market data!R18C2HestonProcess,A</v>
       </c>
       <c r="D98" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="99" spans="1:4">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>53</v>
       </c>
@@ -1848,7 +1811,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="100" spans="1:4">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>59</v>
       </c>
@@ -1856,7 +1819,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="101" spans="1:4">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>63</v>
       </c>
@@ -1867,7 +1830,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="102" spans="1:4">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>65</v>
       </c>
@@ -1875,7 +1838,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="103" spans="1:4">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>67</v>
       </c>
@@ -1883,7 +1846,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="104" spans="1:4">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>69</v>
       </c>
@@ -1894,7 +1857,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="105" spans="1:4">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>77</v>
       </c>
@@ -1902,7 +1865,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="106" spans="1:4">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>79</v>
       </c>
@@ -1910,7 +1873,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="107" spans="1:4">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>61</v>
       </c>
@@ -1918,40 +1881,40 @@
         <v>62</v>
       </c>
     </row>
-    <row r="109" spans="1:4">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>81</v>
       </c>
-      <c r="B109" s="2" t="e">
-        <f t="array" aca="1" ref="B109" ca="1">_xll.qlMCDiscreteArithmeticAPHestonEngine(B98,B99,,B101,,,B104,,,,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4">
+      <c r="B109" s="2" t="str">
+        <f t="array" ref="B109">_xll.qlMCDiscreteArithmeticAPHestonEngine(B98,B99,,B101,,,B104,,,,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R109C2MCLDDiscreteArithmeticAPHestonEngine,A</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>24</v>
       </c>
-      <c r="B110" s="6" t="e">
-        <f t="array" aca="1" ref="B110" ca="1">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B109))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4">
+      <c r="B110" s="6">
+        <f t="array" ref="B110">_xll.qlInstrumentNPV($B$39,_xll.qlInstrumentSetPricingEngine($B$39,B109))</f>
+        <v>6.4452596351224285</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>82</v>
       </c>
-      <c r="B112" s="2" t="e">
-        <f t="array" aca="1" ref="B112" ca="1">_xll.qlMCDiscreteGeometricAPHestonEngine(B98,B99,,B101,,,B104,,,B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2">
+      <c r="B112" s="2" t="str">
+        <f t="array" ref="B112">_xll.qlMCDiscreteGeometricAPHestonEngine(B98,B99,,B101,,,B104,,,B1)</f>
+        <v>欣[test_asianoptions.xlsx]DiscreteAveragingAsianOption!R112C2MCLDDiscreteGeometricAPHestonEngine,A</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>24</v>
       </c>
-      <c r="B113" s="6" t="e">
-        <f t="array" aca="1" ref="B113" ca="1">_xll.qlInstrumentNPV($B$34,_xll.qlInstrumentSetPricingEngine($B$34,B112))</f>
-        <v>#VALUE!</v>
+      <c r="B113" s="6">
+        <f t="array" ref="B113">_xll.qlInstrumentNPV($B$34,_xll.qlInstrumentSetPricingEngine($B$34,B112))</f>
+        <v>5.6541859159431116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>